<commit_message>
Added changes in dev data json and agent factory.
</commit_message>
<xml_diff>
--- a/scripts/Voice_Test_Matrix.xlsx
+++ b/scripts/Voice_Test_Matrix.xlsx
@@ -532,10 +532,24 @@
           <t>Brooke - Big Sister</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>475</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>+19894742667</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>LLM never responded, TTS only produced 5 chars (greeting only)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -564,9 +578,19 @@
           <t>Katie - Friendly Fixer</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>466</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>+16827328687</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="n"/>
     </row>
     <row r="4">
@@ -596,9 +620,19 @@
           <t>Jacqueline - Reassuring Agent</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>468</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>+15076506421</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="n"/>
     </row>
     <row r="5">
@@ -628,10 +662,24 @@
           <t>Autumn</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>467</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>+17405204895</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>TTS produced no audio (0 tts_usage entries)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -660,10 +708,24 @@
           <t>Fahad</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>471</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>+12183093029</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>TTS produced no audio (0 tts_usage entries)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -692,9 +754,19 @@
           <t>Expressive Narrator</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>472</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>+16562614918</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="n"/>
     </row>
     <row r="8">
@@ -724,9 +796,19 @@
           <t>Radiant Girl</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>470</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>+13186201704</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="n"/>
     </row>
     <row r="9">
@@ -756,9 +838,19 @@
           <t>Magnetic-voiced Male</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>473</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>+12763881949</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="n"/>
     </row>
     <row r="10">
@@ -788,9 +880,19 @@
           <t>Compelling Lady</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>469</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>+13186682645</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="n"/>
     </row>
     <row r="11">
@@ -820,9 +922,19 @@
           <t>Aussie Bloke</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>474</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>+13187133023</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="n"/>
     </row>
     <row r="12">
@@ -852,9 +964,19 @@
           <t>Captivating Female</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>481</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>+19894742667</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="n"/>
     </row>
     <row r="13">
@@ -884,9 +1006,19 @@
           <t>albion</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>476</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>+16827328687</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="n"/>
     </row>
     <row r="14">
@@ -916,9 +1048,19 @@
           <t>astra</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>478</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>+15076506421</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="n"/>
     </row>
     <row r="15">
@@ -948,9 +1090,19 @@
           <t>alexis</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>477</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>+17405204895</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="n"/>
     </row>
     <row r="16">
@@ -1044,9 +1196,19 @@
           <t>Ashley</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>479</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>+13186201704</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="n"/>
     </row>
     <row r="19">
@@ -1076,9 +1238,19 @@
           <t>Alex</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>480</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>+12763881949</t>
+        </is>
+      </c>
       <c r="J19" s="2" t="n"/>
     </row>
     <row r="20">
@@ -1204,9 +1376,19 @@
           <t>Abhi</t>
         </is>
       </c>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>486</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>+16562614918</t>
+        </is>
+      </c>
       <c r="J23" s="2" t="n"/>
     </row>
     <row r="24">
@@ -1236,9 +1418,19 @@
           <t>Ava</t>
         </is>
       </c>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>482</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>+13186201704</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="n"/>
     </row>
     <row r="25">
@@ -1268,9 +1460,19 @@
           <t>Colton Rivers</t>
         </is>
       </c>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>484</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>+12763881949</t>
+        </is>
+      </c>
       <c r="J25" s="2" t="n"/>
     </row>
     <row r="26">
@@ -1300,9 +1502,19 @@
           <t>Dungeon Master</t>
         </is>
       </c>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>483</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>+13186682645</t>
+        </is>
+      </c>
       <c r="J26" s="2" t="n"/>
     </row>
     <row r="27">
@@ -1332,9 +1544,19 @@
           <t>Roger - Laid-Back, Casual, Resonant</t>
         </is>
       </c>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>485</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>+13187133023</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="n"/>
     </row>
     <row r="28">
@@ -1364,9 +1586,19 @@
           <t>Sarah - Mature, Reassuring, Confident</t>
         </is>
       </c>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="n"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>490</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>+16562614918</t>
+        </is>
+      </c>
       <c r="J28" s="2" t="n"/>
     </row>
     <row r="29">
@@ -1396,9 +1628,19 @@
           <t>Laura - Enthusiast, Quirky Attitude</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>487</v>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>+13186201704</t>
+        </is>
+      </c>
       <c r="J29" s="2" t="n"/>
     </row>
     <row r="30">
@@ -1428,9 +1670,19 @@
           <t>Charlie - Deep, Confident, Energetic</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>489</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>+12763881949</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="n"/>
     </row>
     <row r="31">
@@ -1460,9 +1712,19 @@
           <t>Pirate Captain</t>
         </is>
       </c>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>488</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>+13186682645</t>
+        </is>
+      </c>
       <c r="J31" s="2" t="n"/>
     </row>
     <row r="32">
@@ -1492,9 +1754,19 @@
           <t>British Butler</t>
         </is>
       </c>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>491</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>+13187133023</t>
+        </is>
+      </c>
       <c r="J32" s="2" t="n"/>
     </row>
     <row r="33">
@@ -1524,9 +1796,19 @@
           <t>Cartoon Villain</t>
         </is>
       </c>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>495</v>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>+16562614918</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="n"/>
     </row>
     <row r="34">
@@ -1556,9 +1838,19 @@
           <t>Medieval Knight</t>
         </is>
       </c>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>492</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>+13186201704</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="n"/>
     </row>
     <row r="35">
@@ -1588,9 +1880,19 @@
           <t>Nyomi</t>
         </is>
       </c>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>496</v>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>+12763881949</t>
+        </is>
+      </c>
       <c r="J35" s="2" t="n"/>
     </row>
     <row r="36">
@@ -1620,9 +1922,19 @@
           <t>Sarah</t>
         </is>
       </c>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>493</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>+13186682645</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="n"/>
     </row>
   </sheetData>

</xml_diff>